<commit_message>
Corrigido detalhes das telas de mercado corrigido erros de imagem, e modulando telas de carteira e da conta.
</commit_message>
<xml_diff>
--- a/docs/startups_mescla_invest.xlsx
+++ b/docs/startups_mescla_invest.xlsx
@@ -484,48 +484,43 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AgroVision AI</t>
+          <t>BioGrid Solutions</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Plataforma que utiliza visão computacional e IA para monitoramento de plantações, identificando pragas e falhas no cultivo em tempo real via drones.</t>
+          <t>Transformamos lixo orgânico em eletricidade e fertilizantes através de biodigestores modulares.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Em operação</t>
+          <t>Nova</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Agrotech</t>
+          <t>CleanTech / Energia</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>250000</v>
+        <v>450062</v>
       </c>
       <c r="G2" t="n">
-        <v>1000000</v>
+        <v>1000</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Lucas Andrade; Fernanda Costa</t>
+          <t>Ricardo Gomes</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>60; 40</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Dr. Roberto Lima; Ana Souza</t>
+          <t>70</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://example.com/agrovision-demo</t>
+          <t>startups/3T6WbL2zAqFLL26ehGvU/video.mp4</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -540,48 +535,48 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HealthChain</t>
+          <t>SolarStream</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sistema de prontuários médicos descentralizados utilizando blockchain, garantindo segurança e interoperabilidade entre clínicas e hospitais.</t>
+          <t>Aluguel de painéis solares remotos com desconto direto na conta de luz via app.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Em expansão</t>
+          <t>Em operação</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Healthtech</t>
+          <t>Energy / Sustentabilidade</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>500000</v>
+        <v>1200123</v>
       </c>
       <c r="G3" t="n">
-        <v>2000000</v>
+        <v>500</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Mariana Alves; Carlos Mendes; João Ribeiro</t>
+          <t>Ana Clara</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>40; 35; 25</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Dra. Paula Martins; Ricardo Teixeira</t>
+          <t>Paulo Guedes</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://example.com/healthchain-demo</t>
+          <t>startups/AATXPQHFdO74vCAlVeHG/video.mp4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -596,48 +591,43 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EduFlex</t>
+          <t>QuantumSec</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Plataforma de microlearning adaptativo com trilhas personalizadas baseadas em IA para estudantes universitários.</t>
+          <t>Proteção de dados governamentais e bancários contra ataques de computação quântica.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Nova</t>
+          <t>Em expansão</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Edtech</t>
+          <t>Cybersecurity / Quantum</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>80000</v>
+        <v>5800000</v>
       </c>
       <c r="G4" t="n">
-        <v>500000</v>
+        <v>200</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Beatriz Rocha</t>
+          <t>Dr. Helena Wu</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Prof. André Silva</t>
+          <t>35</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://example.com/eduflex-demo</t>
+          <t>startups/SCXonYzWO8w9sNc9agUI/video.mp4</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -652,12 +642,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UrbanMob</t>
+          <t>OceanPurify</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Aplicativo de mobilidade urbana focado em rotas inteligentes e integração entre transporte público e privado.</t>
+          <t>Utilizamos drones subaquáticos inteligentes para mapear e remover detritos plásticos de oceanos e rios.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -667,33 +657,33 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Mobility</t>
+          <t>OceanTech / Sustentabilidade</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>300000</v>
+        <v>3200003</v>
       </c>
       <c r="G5" t="n">
-        <v>1200000</v>
+        <v>650</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Rafael Gomes; Juliana Martins</t>
+          <t>Marina Lopez</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>55; 45</t>
+          <t>45</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Eduardo Nunes; Patrícia Lima</t>
+          <t>Jean Cousteau</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://example.com/urbanmob-demo</t>
+          <t>startups/gDCWCetvJiUTpFP11EsG/video.mp4</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -708,12 +698,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GreenEnergy Token</t>
+          <t>AgroMind AI</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Plataforma de financiamento coletivo para projetos de energia renovável com tokenização de participação em usinas solares.</t>
+          <t>Plataforma baseada em IA e visão computacional para monitorar plantações em tempo real, prever pragas e otimizar irrigação através de drones e sensores IoT.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -723,33 +713,33 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Energy / Cleantech</t>
+          <t>AgTech / AI / IoT</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>750000</v>
+        <v>845000</v>
       </c>
       <c r="G6" t="n">
-        <v>3000000</v>
+        <v>1200</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Thiago Pereira; Camila Fernandes; Bruno Lopes</t>
+          <t>Lucas Andrade; Fernanda Costa</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>34; 33; 33</t>
+          <t>55; 45</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Eng. Marcos Silva; Laura Dias</t>
+          <t>Marcos Vieira</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://example.com/greenenergy-demo</t>
+          <t>startups/agromind-ai/video.mp4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">

</xml_diff>